<commit_message>
SPM-77: Kayalvizhi's test run after the review fixes (TC01-TC15 pass)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-77_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-77_Test_Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krist\Documents\GitHub\IS212\docs\test-cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\IS212\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2AE4A2-78FA-4ABC-8AE8-CC377C02E580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDE8E1A6-29B8-4619-9944-83F2D3EC578B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14715" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10070" yWindow="0" windowWidth="9220" windowHeight="10170" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="183">
   <si>
     <t>Item</t>
   </si>
@@ -817,6 +817,12 @@
 Step 4: The list offers 'Podium Light — Staging' (requested only for Day 2). It offers neither Ring Light nor Portable Stage, which Day 1 already requests.
 Step 5: '4 available for these dates — enough for this suggestion.' appears under 'Quantity'.
 Step 7: The form closes. 'Suggestion sent to the Coordinator.' appears on the Ring Light line, which now reads 'Suggested alternative: 4 × Podium Light — waiting for the Coordinator's decision.' The Day 2 Podium Light line is unchanged.</t>
+  </si>
+  <si>
+    <t>ccb81a8</t>
+  </si>
+  <si>
+    <t>Kayalvizhi</t>
   </si>
 </sst>
 </file>
@@ -1029,22 +1035,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1262,7 +1268,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I32"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1275,22 +1281,22 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>22</v>
       </c>
       <c r="B1" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="18"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="19"/>
+    </row>
+    <row r="3" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>24</v>
       </c>
@@ -1319,7 +1325,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>32</v>
       </c>
@@ -1344,7 +1350,7 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
     </row>
-    <row r="5" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>39</v>
       </c>
@@ -1369,7 +1375,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
     </row>
-    <row r="6" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>43</v>
       </c>
@@ -1394,7 +1400,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
     </row>
-    <row r="7" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>48</v>
       </c>
@@ -1419,7 +1425,7 @@
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
     </row>
-    <row r="8" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>52</v>
       </c>
@@ -1469,7 +1475,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>60</v>
       </c>
@@ -1519,7 +1525,7 @@
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
     </row>
-    <row r="12" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>69</v>
       </c>
@@ -1569,7 +1575,7 @@
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
     </row>
-    <row r="14" spans="1:9" ht="52.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="52.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>77</v>
       </c>
@@ -1594,7 +1600,7 @@
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
     </row>
-    <row r="15" spans="1:9" ht="52.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="52.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>82</v>
       </c>
@@ -1619,7 +1625,7 @@
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:9" ht="52.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="52.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>86</v>
       </c>
@@ -1644,7 +1650,7 @@
       <c r="H16" s="9"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="17" spans="1:9" ht="52.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="52.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>89</v>
       </c>
@@ -1669,7 +1675,7 @@
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
     </row>
-    <row r="18" spans="1:9" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="39.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>93</v>
       </c>
@@ -1694,163 +1700,169 @@
       <c r="H18" s="9"/>
       <c r="I18" s="9"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="13" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>94</v>
       </c>
       <c r="B21" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="C21" s="19"/>
-      <c r="D21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
       <c r="E21" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="F21" s="18"/>
-    </row>
-    <row r="22" spans="1:9" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="19"/>
+    </row>
+    <row r="22" spans="1:9" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>92</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="19"/>
       <c r="E22" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="F22" s="18"/>
-    </row>
-    <row r="23" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="19"/>
+    </row>
+    <row r="23" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>99</v>
       </c>
       <c r="B23" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="19"/>
       <c r="E23" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="F23" s="18"/>
-    </row>
-    <row r="24" spans="1:9" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="19"/>
+    </row>
+    <row r="24" spans="1:9" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>102</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C24" s="19"/>
-      <c r="D24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
       <c r="E24" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="F24" s="18"/>
-    </row>
-    <row r="25" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="19"/>
+    </row>
+    <row r="25" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>105</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="C25" s="19"/>
-      <c r="D25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="F25" s="18"/>
-    </row>
-    <row r="26" spans="1:9" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F25" s="19"/>
+    </row>
+    <row r="26" spans="1:9" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>51</v>
       </c>
       <c r="B26" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="19"/>
-      <c r="D26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="19"/>
       <c r="E26" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="F26" s="18"/>
-    </row>
-    <row r="27" spans="1:9" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F26" s="19"/>
+    </row>
+    <row r="27" spans="1:9" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>59</v>
       </c>
       <c r="B27" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="C27" s="19"/>
-      <c r="D27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="19"/>
       <c r="E27" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F27" s="18"/>
-    </row>
-    <row r="28" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F27" s="19"/>
+    </row>
+    <row r="28" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>111</v>
       </c>
       <c r="B28" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="C28" s="19"/>
-      <c r="D28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="19"/>
       <c r="E28" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="F28" s="18"/>
-    </row>
-    <row r="29" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F28" s="19"/>
+    </row>
+    <row r="29" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
         <v>113</v>
       </c>
       <c r="B29" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="19"/>
       <c r="E29" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="F29" s="18"/>
-    </row>
-    <row r="30" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F29" s="19"/>
+    </row>
+    <row r="30" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>72</v>
       </c>
       <c r="B30" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="19"/>
       <c r="E30" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F30" s="18"/>
-    </row>
-    <row r="32" spans="1:9" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F30" s="19"/>
+    </row>
+    <row r="32" spans="1:9" ht="166" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>118</v>
       </c>
       <c r="B32" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="E28:F28"/>
     <mergeCell ref="B32:I32"/>
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="B30:D30"/>
@@ -1867,12 +1879,6 @@
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="E24:F24"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="E28:F28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'TC01'!A1" display="TC01" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -1897,20 +1903,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -1918,7 +1924,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -1926,7 +1932,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -1934,7 +1940,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="184.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="184.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -1942,7 +1948,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -1950,7 +1956,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -1958,7 +1964,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -1966,7 +1972,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -1974,14 +1980,14 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="118.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="118.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -1989,7 +1995,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -1997,7 +2003,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2005,7 +2011,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -2013,7 +2019,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2021,12 +2027,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="121.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2039,20 +2101,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2060,7 +2122,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2068,7 +2130,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2076,7 +2138,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2084,7 +2146,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2092,7 +2154,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2100,7 +2162,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2108,7 +2170,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2116,14 +2178,14 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="118.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="118.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2131,7 +2193,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2139,7 +2201,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2147,7 +2209,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -2155,7 +2217,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2163,12 +2225,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="102.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2181,20 +2299,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="74.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:3" ht="74.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="24"/>
-    </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="22"/>
+    </row>
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2202,7 +2320,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2210,7 +2328,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2218,7 +2336,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2226,7 +2344,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2234,7 +2352,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2242,7 +2360,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2250,7 +2368,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2258,14 +2376,14 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="145.19999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="145.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2273,7 +2391,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2281,7 +2399,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2289,7 +2407,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -2297,7 +2415,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2305,12 +2423,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="116" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2326,20 +2500,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="22"/>
-    </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="24"/>
+    </row>
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2347,7 +2521,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2355,7 +2529,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2363,7 +2537,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2371,7 +2545,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2379,7 +2553,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2387,7 +2561,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2395,7 +2569,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2403,7 +2577,7 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -2418,7 +2592,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2426,7 +2600,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2434,7 +2608,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -2442,7 +2616,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2450,12 +2624,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="144.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2471,20 +2701,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:3" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="22"/>
-    </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="24"/>
+    </row>
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2492,7 +2722,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2500,7 +2730,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2508,7 +2738,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2516,7 +2746,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2524,7 +2754,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="243.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="243.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2532,7 +2762,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2540,7 +2770,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2548,7 +2778,7 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -2563,7 +2793,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2571,7 +2801,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2579,7 +2809,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -2587,7 +2817,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2595,12 +2825,68 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>176</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="236" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2616,20 +2902,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2637,7 +2923,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2645,7 +2931,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2653,7 +2939,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="118.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="118.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2661,7 +2947,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2669,7 +2955,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="189" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2677,7 +2963,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2685,7 +2971,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2693,14 +2979,14 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="195.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="195.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -2708,7 +2994,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2716,7 +3002,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2724,7 +3010,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -2732,7 +3018,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2740,12 +3026,68 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>176</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="183" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2758,20 +3100,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2779,7 +3121,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2787,7 +3129,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2795,7 +3137,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2803,7 +3145,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2811,7 +3153,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2819,7 +3161,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2827,7 +3169,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2835,7 +3177,7 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -2850,7 +3192,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2858,7 +3200,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -2866,7 +3208,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -2874,7 +3216,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -2882,13 +3224,67 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="66" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>ccb81a8</t>
+          <t>dfe3697</t>
         </is>
       </c>
     </row>
@@ -2902,20 +3298,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -2923,7 +3319,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -2931,7 +3327,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -2939,7 +3335,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2947,7 +3343,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -2955,7 +3351,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="301.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="301" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -2963,7 +3359,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -2971,7 +3367,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -2979,7 +3375,7 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -2994,7 +3390,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3002,7 +3398,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -3010,7 +3406,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -3018,7 +3414,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -3026,12 +3422,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="289" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3044,20 +3496,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3065,7 +3517,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3073,7 +3525,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3081,7 +3533,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3089,7 +3541,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3097,7 +3549,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -3105,7 +3557,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3113,7 +3565,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3121,7 +3573,7 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -3136,7 +3588,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3144,7 +3596,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -3152,7 +3604,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -3160,7 +3612,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -3168,12 +3620,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="139.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3186,20 +3694,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3207,7 +3715,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3215,7 +3723,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3223,7 +3731,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3231,7 +3739,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3239,7 +3747,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="193.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -3247,7 +3755,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3255,7 +3763,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3263,14 +3771,14 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="171.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="171.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -3278,7 +3786,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3286,7 +3794,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -3294,7 +3802,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -3302,7 +3810,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -3310,12 +3818,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3328,20 +3892,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3349,7 +3913,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3357,7 +3921,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3365,7 +3929,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="193.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3373,7 +3937,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3381,7 +3945,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="233.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="233.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -3389,7 +3953,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3397,7 +3961,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3405,7 +3969,7 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -3420,7 +3984,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3428,7 +3992,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -3436,7 +4000,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -3444,7 +4008,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -3452,12 +4016,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="228.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3470,20 +4090,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3491,7 +4111,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3499,7 +4119,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3507,7 +4127,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3515,7 +4135,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3523,7 +4143,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -3531,7 +4151,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3539,7 +4159,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3547,7 +4167,7 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -3562,7 +4182,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3570,7 +4190,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -3578,7 +4198,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -3586,7 +4206,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -3594,12 +4214,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="130" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3612,20 +4288,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3633,7 +4309,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3641,7 +4317,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3649,7 +4325,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3657,7 +4333,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3665,7 +4341,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -3673,7 +4349,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3681,7 +4357,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3689,7 +4365,7 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
@@ -3704,7 +4380,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3712,7 +4388,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -3720,7 +4396,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -3728,7 +4404,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -3736,12 +4412,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3754,20 +4486,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3775,7 +4507,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3783,7 +4515,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3791,7 +4523,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3799,7 +4531,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3807,7 +4539,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="247.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="247" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -3815,7 +4547,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3823,7 +4555,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3831,14 +4563,14 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="211.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="211.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -3846,7 +4578,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3854,7 +4586,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -3862,7 +4594,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -3870,7 +4602,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -3878,12 +4610,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="203" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3896,20 +4684,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" customWidth="1"/>
-    <col min="2" max="2" width="56.77734375" customWidth="1"/>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -3917,7 +4705,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
@@ -3925,7 +4713,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -3933,7 +4721,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="193.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -3941,7 +4729,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
@@ -3949,7 +4737,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
@@ -3957,7 +4745,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>13</v>
       </c>
@@ -3965,7 +4753,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>15</v>
       </c>
@@ -3973,14 +4761,14 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="118.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="118.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
@@ -3988,7 +4776,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -3996,7 +4784,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>18</v>
       </c>
@@ -4004,7 +4792,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
@@ -4012,7 +4800,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>20</v>
       </c>
@@ -4020,12 +4808,68 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="5"/>
+    </row>
+    <row r="19" spans="1:2" ht="122" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="12">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>dfe3697</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>